<commit_message>
Cleaning source file programmed
</commit_message>
<xml_diff>
--- a/03_process_editions/Metadata/Editions.xlsx
+++ b/03_process_editions/Metadata/Editions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanniejo\Documents_local\01_dataplatform\021_SVbevraging\01_code\02_process_editions\Metadata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vanniejo\Documents_local\01_dataplatform\021_SVbevraging\01_code\03_process_editions\Metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91136E91-2701-41CE-9D04-C5FA8E640661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B4F558D-BF26-414D-8AF1-D378D942E2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="edities" sheetId="1" r:id="rId1"/>
@@ -33,14 +33,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="33">
   <si>
     <t>cntctprs</t>
   </si>
   <si>
-    <t>SV1</t>
-  </si>
-  <si>
     <t>voorjaar</t>
   </si>
   <si>
@@ -50,21 +47,9 @@
     <t>Homo Sapiens Sapiens (MAS)</t>
   </si>
   <si>
-    <t>SV2-SV3</t>
-  </si>
-  <si>
     <t>najaar</t>
   </si>
   <si>
-    <t>SV4</t>
-  </si>
-  <si>
-    <t>SV5-SV6</t>
-  </si>
-  <si>
-    <t>SV7</t>
-  </si>
-  <si>
     <t>IPSOS</t>
   </si>
   <si>
@@ -95,15 +80,9 @@
     <t>SV0009</t>
   </si>
   <si>
-    <t>SV8-SV9</t>
-  </si>
-  <si>
     <t>SV0010</t>
   </si>
   <si>
-    <t>SV10</t>
-  </si>
-  <si>
     <t>SV0011</t>
   </si>
   <si>
@@ -113,24 +92,15 @@
     <t>SV0012</t>
   </si>
   <si>
-    <t>SV11-SV12</t>
-  </si>
-  <si>
     <t>SV0013</t>
   </si>
   <si>
-    <t>SV13</t>
-  </si>
-  <si>
     <t>SV0014</t>
   </si>
   <si>
     <t>SV0015</t>
   </si>
   <si>
-    <t>SV14-SV15</t>
-  </si>
-  <si>
     <t>surv_id</t>
   </si>
   <si>
@@ -147,6 +117,21 @@
   </si>
   <si>
     <t>fw_org</t>
+  </si>
+  <si>
+    <t>SV0002-SV0003</t>
+  </si>
+  <si>
+    <t>SV0005-SV0006</t>
+  </si>
+  <si>
+    <t>SV0008-SV0009</t>
+  </si>
+  <si>
+    <t>SV0011-SV0012</t>
+  </si>
+  <si>
+    <t>SV0014-SV0015</t>
   </si>
 </sst>
 </file>
@@ -997,383 +982,383 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="F1" t="s">
         <v>0</v>
       </c>
       <c r="G1" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>2021</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>6000</v>
       </c>
       <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
         <v>3</v>
       </c>
-      <c r="G2" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="C3">
         <v>2021</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E3">
         <v>6000</v>
       </c>
       <c r="F3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" t="s">
         <v>3</v>
       </c>
-      <c r="G3" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="C4">
         <v>2021</v>
       </c>
       <c r="D4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E4">
         <v>6000</v>
       </c>
       <c r="F4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" t="s">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>2022</v>
       </c>
       <c r="D5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
         <v>6000</v>
       </c>
       <c r="F5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
         <v>3</v>
       </c>
-      <c r="G5" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C6">
         <v>2022</v>
       </c>
       <c r="D6" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6">
         <v>6000</v>
       </c>
       <c r="F6" t="s">
+        <v>2</v>
+      </c>
+      <c r="G6" t="s">
         <v>3</v>
       </c>
-      <c r="G6" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C7">
         <v>2022</v>
       </c>
       <c r="D7" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E7">
         <v>6000</v>
       </c>
       <c r="F7" t="s">
+        <v>2</v>
+      </c>
+      <c r="G7" t="s">
         <v>3</v>
       </c>
-      <c r="G7" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C8">
         <v>2023</v>
       </c>
       <c r="D8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8">
         <v>6000</v>
       </c>
       <c r="F8" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C9">
         <v>2023</v>
       </c>
       <c r="D9" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E9">
         <v>6000</v>
       </c>
       <c r="F9" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G9" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C10">
         <v>2023</v>
       </c>
       <c r="D10" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E10">
         <v>6000</v>
       </c>
       <c r="F10" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C11">
         <v>2024</v>
       </c>
       <c r="D11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>6000</v>
       </c>
       <c r="F11" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C12">
         <v>2024</v>
       </c>
       <c r="D12" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E12">
         <v>6000</v>
       </c>
       <c r="F12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G12" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C13">
         <v>2024</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E13">
         <v>6000</v>
       </c>
       <c r="F13" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C14">
         <v>2025</v>
       </c>
       <c r="D14" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14">
         <v>6000</v>
       </c>
       <c r="F14" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G14" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C15">
         <v>2025</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E15">
         <v>6000</v>
       </c>
       <c r="F15" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G15" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16">
         <v>2025</v>
       </c>
       <c r="D16" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E16">
         <v>6000</v>
       </c>
       <c r="F16" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1383,6 +1368,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ff9b9dd8-fcc8-4df5-a108-c5866d1d7b9b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9a9ec0f0-7796-43d0-ac1f-4c8c46ee0bd1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A6AD3661E8CB194C8675B85DE5B2CF8E" ma:contentTypeVersion="18" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="74052aabd80d88734f9eb511f320c0f7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ff9b9dd8-fcc8-4df5-a108-c5866d1d7b9b" xmlns:ns3="5b0c7779-fcdd-4d12-9999-ca37719676af" xmlns:ns4="9a9ec0f0-7796-43d0-ac1f-4c8c46ee0bd1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c4265b27bfda865713f908aeb805a5eb" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="ff9b9dd8-fcc8-4df5-a108-c5866d1d7b9b"/>
@@ -1630,17 +1626,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ff9b9dd8-fcc8-4df5-a108-c5866d1d7b9b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9a9ec0f0-7796-43d0-ac1f-4c8c46ee0bd1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1651,6 +1636,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70B9D0FF-9A62-4395-A00E-55F7A309D652}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="ff9b9dd8-fcc8-4df5-a108-c5866d1d7b9b"/>
+    <ds:schemaRef ds:uri="9a9ec0f0-7796-43d0-ac1f-4c8c46ee0bd1"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01888A4F-88AC-4929-924A-5D35044FC667}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1670,17 +1666,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{70B9D0FF-9A62-4395-A00E-55F7A309D652}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ff9b9dd8-fcc8-4df5-a108-c5866d1d7b9b"/>
-    <ds:schemaRef ds:uri="9a9ec0f0-7796-43d0-ac1f-4c8c46ee0bd1"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{34D17C01-2DE4-45DF-8872-FEC3D25CEFE2}">
   <ds:schemaRefs>

</xml_diff>